<commit_message>
añadiendo detalles de numeros 5, matriz de confusion, boxplot
</commit_message>
<xml_diff>
--- a/out/global_metric/excel/alexnet.xlsx
+++ b/out/global_metric/excel/alexnet.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,15 +446,35 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>tn</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>fp</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>fn</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>tp</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>model</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>fold</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>submodel</t>
         </is>
@@ -465,20 +485,32 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.9583333333333334</v>
+        <v>0.9583333134651184</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8357142757500001</v>
-      </c>
-      <c r="D2" t="inlineStr">
+        <v>0.9559599993740974</v>
+      </c>
+      <c r="D2" t="n">
+        <v>61</v>
+      </c>
+      <c r="E2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>alexnet</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="I2" t="n">
         <v>0</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
@@ -489,20 +521,32 @@
         <v>19</v>
       </c>
       <c r="B3" t="n">
-        <v>0.9285714285714286</v>
+        <v>0.9404761791229248</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7214285627261905</v>
-      </c>
-      <c r="D3" t="inlineStr">
+        <v>0.9368990333437516</v>
+      </c>
+      <c r="D3" t="n">
+        <v>59</v>
+      </c>
+      <c r="E3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" t="n">
+        <v>99</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>alexnet</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="I3" t="n">
         <v>1</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
@@ -513,20 +557,32 @@
         <v>38</v>
       </c>
       <c r="B4" t="n">
-        <v>0.9464285714285716</v>
+        <v>0.9464285969734192</v>
       </c>
       <c r="C4" t="n">
-        <v>0.7733559998540385</v>
-      </c>
-      <c r="D4" t="inlineStr">
+        <v>0.9418796796871874</v>
+      </c>
+      <c r="D4" t="n">
+        <v>56</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>8</v>
+      </c>
+      <c r="G4" t="n">
+        <v>103</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>alexnet</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="I4" t="n">
         <v>2</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
@@ -537,20 +593,32 @@
         <v>57</v>
       </c>
       <c r="B5" t="n">
-        <v>0.9226190476190474</v>
+        <v>0.9404761791229248</v>
       </c>
       <c r="C5" t="n">
-        <v>0.7408163181093296</v>
-      </c>
-      <c r="D5" t="inlineStr">
+        <v>0.9368990333437516</v>
+      </c>
+      <c r="D5" t="n">
+        <v>59</v>
+      </c>
+      <c r="E5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G5" t="n">
+        <v>99</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>alexnet</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="I5" t="n">
         <v>3</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
@@ -561,140 +629,32 @@
         <v>76</v>
       </c>
       <c r="B6" t="n">
-        <v>0.9404761904761902</v>
+        <v>0.9345238208770752</v>
       </c>
       <c r="C6" t="n">
-        <v>0.8293650693485451</v>
-      </c>
-      <c r="D6" t="inlineStr">
+        <v>0.9303771187951062</v>
+      </c>
+      <c r="D6" t="n">
+        <v>58</v>
+      </c>
+      <c r="E6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>6</v>
+      </c>
+      <c r="G6" t="n">
+        <v>99</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>alexnet</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="I6" t="n">
         <v>4</v>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>95</v>
-      </c>
-      <c r="B7" t="n">
-        <v>0.9285714285714286</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0.7535147304558903</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>alexnet</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>5</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>114</v>
-      </c>
-      <c r="B8" t="n">
-        <v>0.9107142857142856</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0.7331065672067814</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>alexnet</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>6</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>133</v>
-      </c>
-      <c r="B9" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0.757142848559524</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>alexnet</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>7</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>152</v>
-      </c>
-      <c r="B10" t="n">
-        <v>0.9583333333333334</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0.8134920537367725</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>alexnet</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>8</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>171</v>
-      </c>
-      <c r="B11" t="n">
-        <v>0.886904761904762</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0.7100906949303263</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>alexnet</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>9</v>
-      </c>
-      <c r="F11" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>nan</t>
         </is>

</xml_diff>

<commit_message>
modifications to quit the stars
</commit_message>
<xml_diff>
--- a/out/global_metric/excel/alexnet.xlsx
+++ b/out/global_metric/excel/alexnet.xlsx
@@ -495,28 +495,28 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.9523809552192688</v>
+        <v>0.8404074907302856</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9495192256497608</v>
+        <v>0.8394704440626617</v>
       </c>
       <c r="D2" t="n">
-        <v>60</v>
+        <v>225</v>
       </c>
       <c r="E2" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="F2" t="n">
-        <v>4</v>
+        <v>69</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>270</v>
       </c>
       <c r="H2" t="n">
-        <v>0.9918118990384616</v>
+        <v>0.9150466966447596</v>
       </c>
       <c r="I2" t="n">
-        <v>0.9948768065547222</v>
+        <v>0.904114647812876</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -537,28 +537,28 @@
         <v>23</v>
       </c>
       <c r="B3" t="n">
-        <v>0.9047619104385376</v>
+        <v>0.833616316318512</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9011764654900072</v>
+        <v>0.8330923635354294</v>
       </c>
       <c r="D3" t="n">
-        <v>60</v>
+        <v>229</v>
       </c>
       <c r="E3" t="n">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="F3" t="n">
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="G3" t="n">
-        <v>92</v>
+        <v>262</v>
       </c>
       <c r="H3" t="n">
-        <v>0.9813701923076924</v>
+        <v>0.9110169491525424</v>
       </c>
       <c r="I3" t="n">
-        <v>0.9894130216522116</v>
+        <v>0.8998227451469347</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -579,28 +579,28 @@
         <v>46</v>
       </c>
       <c r="B4" t="n">
-        <v>0.9464285969734192</v>
+        <v>0.8217317461967468</v>
       </c>
       <c r="C4" t="n">
-        <v>0.9436976303337532</v>
+        <v>0.8209866308628972</v>
       </c>
       <c r="D4" t="n">
-        <v>61</v>
+        <v>223</v>
       </c>
       <c r="E4" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>72</v>
       </c>
       <c r="G4" t="n">
-        <v>98</v>
+        <v>261</v>
       </c>
       <c r="H4" t="n">
-        <v>0.9914362980769232</v>
+        <v>0.9023175371843652</v>
       </c>
       <c r="I4" t="n">
-        <v>0.9950731146663868</v>
+        <v>0.8854947079501284</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -621,28 +621,28 @@
         <v>69</v>
       </c>
       <c r="B5" t="n">
-        <v>0.9464285969734192</v>
+        <v>0.8353140950202942</v>
       </c>
       <c r="C5" t="n">
-        <v>0.942672980664324</v>
+        <v>0.8353121878017511</v>
       </c>
       <c r="D5" t="n">
-        <v>58</v>
+        <v>247</v>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>50</v>
       </c>
       <c r="F5" t="n">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="G5" t="n">
-        <v>101</v>
+        <v>245</v>
       </c>
       <c r="H5" t="n">
-        <v>0.9729567307692308</v>
+        <v>0.9077135939121412</v>
       </c>
       <c r="I5" t="n">
-        <v>0.9724656747420832</v>
+        <v>0.8956067778789059</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -663,28 +663,28 @@
         <v>92</v>
       </c>
       <c r="B6" t="n">
-        <v>0.9345238208770752</v>
+        <v>0.8200339674949646</v>
       </c>
       <c r="C6" t="n">
-        <v>0.931553015371729</v>
+        <v>0.8200292819385323</v>
       </c>
       <c r="D6" t="n">
-        <v>61</v>
+        <v>240</v>
       </c>
       <c r="E6" t="n">
-        <v>8</v>
+        <v>51</v>
       </c>
       <c r="F6" t="n">
-        <v>3</v>
+        <v>55</v>
       </c>
       <c r="G6" t="n">
-        <v>96</v>
+        <v>243</v>
       </c>
       <c r="H6" t="n">
-        <v>0.9797175480769232</v>
+        <v>0.9067104808024904</v>
       </c>
       <c r="I6" t="n">
-        <v>0.9815387240366508</v>
+        <v>0.8888356189793565</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
adding the another section, the infection
</commit_message>
<xml_diff>
--- a/out/global_metric/excel/alexnet.xlsx
+++ b/out/global_metric/excel/alexnet.xlsx
@@ -495,28 +495,28 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.8404074907302856</v>
+        <v>0.8658743500709534</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8394704440626617</v>
+        <v>0.8658356854287981</v>
       </c>
       <c r="D2" t="n">
-        <v>225</v>
+        <v>250</v>
       </c>
       <c r="E2" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="F2" t="n">
-        <v>69</v>
+        <v>44</v>
       </c>
       <c r="G2" t="n">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="H2" t="n">
-        <v>0.9150466966447596</v>
+        <v>0.9312982820246742</v>
       </c>
       <c r="I2" t="n">
-        <v>0.904114647812876</v>
+        <v>0.9195081227819156</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -537,28 +537,28 @@
         <v>23</v>
       </c>
       <c r="B3" t="n">
-        <v>0.833616316318512</v>
+        <v>0.8641765713691711</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8330923635354294</v>
+        <v>0.8636952648198774</v>
       </c>
       <c r="D3" t="n">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="E3" t="n">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="F3" t="n">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="G3" t="n">
-        <v>262</v>
+        <v>272</v>
       </c>
       <c r="H3" t="n">
-        <v>0.9110169491525424</v>
+        <v>0.9436181252161882</v>
       </c>
       <c r="I3" t="n">
-        <v>0.8998227451469347</v>
+        <v>0.9362229383701132</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -579,28 +579,28 @@
         <v>46</v>
       </c>
       <c r="B4" t="n">
-        <v>0.8217317461967468</v>
+        <v>0.8692699670791626</v>
       </c>
       <c r="C4" t="n">
-        <v>0.8209866308628972</v>
+        <v>0.8688328728079091</v>
       </c>
       <c r="D4" t="n">
-        <v>223</v>
+        <v>239</v>
       </c>
       <c r="E4" t="n">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="F4" t="n">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="G4" t="n">
-        <v>261</v>
+        <v>273</v>
       </c>
       <c r="H4" t="n">
-        <v>0.9023175371843652</v>
+        <v>0.9391502363657328</v>
       </c>
       <c r="I4" t="n">
-        <v>0.8854947079501284</v>
+        <v>0.9360038264601632</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -621,28 +621,28 @@
         <v>69</v>
       </c>
       <c r="B5" t="n">
-        <v>0.8353140950202942</v>
+        <v>0.8471986651420593</v>
       </c>
       <c r="C5" t="n">
-        <v>0.8353121878017511</v>
+        <v>0.8471453236930271</v>
       </c>
       <c r="D5" t="n">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="E5" t="n">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="F5" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="G5" t="n">
-        <v>245</v>
+        <v>255</v>
       </c>
       <c r="H5" t="n">
-        <v>0.9077135939121412</v>
+        <v>0.9304162342903264</v>
       </c>
       <c r="I5" t="n">
-        <v>0.8956067778789059</v>
+        <v>0.923126850067134</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -663,28 +663,28 @@
         <v>92</v>
       </c>
       <c r="B6" t="n">
-        <v>0.8200339674949646</v>
+        <v>0.8862478733062744</v>
       </c>
       <c r="C6" t="n">
-        <v>0.8200292819385323</v>
+        <v>0.8861165651119793</v>
       </c>
       <c r="D6" t="n">
-        <v>240</v>
+        <v>251</v>
       </c>
       <c r="E6" t="n">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="F6" t="n">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="G6" t="n">
-        <v>243</v>
+        <v>271</v>
       </c>
       <c r="H6" t="n">
-        <v>0.9067104808024904</v>
+        <v>0.9559091433183442</v>
       </c>
       <c r="I6" t="n">
-        <v>0.8888356189793565</v>
+        <v>0.9539014988948402</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>

</xml_diff>